<commit_message>
BE-Update project landing page
</commit_message>
<xml_diff>
--- a/public/template/template_Import_Data_TagNumber.xlsx
+++ b/public/template/template_Import_Data_TagNumber.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\project_ta\mechanical_completion_frontend\public\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95BD6C4B-3399-4EEE-B59F-BAE2B5C22465}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B96BDD6-3891-4E6D-BC29-C1F9BA0AF00F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="11625" xr2:uid="{FD925BEE-3942-4A66-984E-78158311B820}"/>
+    <workbookView xWindow="2685" yWindow="2685" windowWidth="21600" windowHeight="11295" xr2:uid="{FD925BEE-3942-4A66-984E-78158311B820}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -232,7 +232,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -252,6 +252,14 @@
       <u/>
       <sz val="11"/>
       <color theme="7"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FFFFC000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -278,13 +286,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -416,7 +425,7 @@
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{10001554-823F-40AC-B388-2AA4C0557914}" name="Table1" displayName="Table1" ref="A1:P29" totalsRowShown="0" dataDxfId="16">
   <autoFilter ref="A1:P29" xr:uid="{7453B12E-FEFF-499F-B9AD-D7D8E87E65E6}"/>
-  <sortState ref="A2:P29">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P29">
     <sortCondition ref="G1:G29"/>
   </sortState>
   <tableColumns count="16">
@@ -760,22 +769,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
       <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>41</v>
       </c>
       <c r="G1" t="s">
@@ -787,13 +796,13 @@
       <c r="I1" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="4" t="s">
         <v>9</v>
       </c>
       <c r="M1" s="3" t="s">

</xml_diff>